<commit_message>
Use stocked equivalent capacitors and OVP resistor for BOM R1
</commit_message>
<xml_diff>
--- a/hardware/kicad/HMT500(ED260313A)/HMT500(ED260313A)_parts_list.xlsx
+++ b/hardware/kicad/HMT500(ED260313A)/HMT500(ED260313A)_parts_list.xlsx
@@ -2211,12 +2211,12 @@
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="H16" s="17" t="inlineStr">
         <is>
-          <t>GRM188R72A102KA01D</t>
+          <t>CL10B102KC8NNNC</t>
         </is>
       </c>
       <c r="I16" s="17" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>C97897</t>
+          <t>C153291</t>
         </is>
       </c>
       <c r="P16" s="16" t="inlineStr">
@@ -3919,12 +3919,12 @@
       </c>
       <c r="G40" s="16" t="inlineStr">
         <is>
-          <t>CAL-CHIP</t>
+          <t>UNI-ROYAL</t>
         </is>
       </c>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>RM06F3652CT</t>
+          <t>0603WAF3652T5E</t>
         </is>
       </c>
       <c r="I40" s="17" t="inlineStr">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>C4027587</t>
+          <t>C23029</t>
         </is>
       </c>
       <c r="P40" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Revise protection resistors for stocked JLC BOM R2
</commit_message>
<xml_diff>
--- a/hardware/kicad/HMT500(ED260313A)/HMT500(ED260313A)_parts_list.xlsx
+++ b/hardware/kicad/HMT500(ED260313A)/HMT500(ED260313A)_parts_list.xlsx
@@ -3621,7 +3621,7 @@
       </c>
       <c r="E36" s="16" t="inlineStr">
         <is>
-          <t>4.7R 1W pulse</t>
+          <t>4.7R 1W 5%</t>
         </is>
       </c>
       <c r="F36" s="16" t="inlineStr">
@@ -3631,17 +3631,17 @@
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>CRCW25124R70FKEG</t>
+          <t>RC2512JK-074R7L</t>
         </is>
       </c>
       <c r="I36" s="17" t="inlineStr">
         <is>
-          <t>CRCW 2512 4.7 Ω 1% 1 W (결정 #38: JLC 부품 — 펄스 내성 HP형 대신 일반형, 서지 시험 T1로 확인) [LCSC: 결정 #38: 일반형 (HP 대신)]</t>
+          <t>YAGEO RC 2512 4.7 Ω 5% 1 W (일반형; 단시간 과부하 원문 확인, 실제 서지 T1 확인 필요) [LCSC: 결정 #57: 일반형 5%; 서지 시험 필요]</t>
         </is>
       </c>
       <c r="J36" s="19" t="n">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>C242563</t>
+          <t>C878295</t>
         </is>
       </c>
       <c r="P36" s="16" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
-          <t>866k 1%</t>
+          <t>845k 1%</t>
         </is>
       </c>
       <c r="F38" s="16" t="inlineStr">
@@ -3775,17 +3775,17 @@
       </c>
       <c r="G38" s="16" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H38" s="17" t="inlineStr">
         <is>
-          <t>RCS0603866KFKEA</t>
+          <t>RC0603FR-07845KL</t>
         </is>
       </c>
       <c r="I38" s="17" t="inlineStr">
         <is>
-          <t>저항 866 kΩ 1% 0603 (UVLO)</t>
+          <t>저항 845 kΩ 1% 0603 (UVLO)</t>
         </is>
       </c>
       <c r="J38" s="19" t="n">
@@ -3809,7 +3809,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>C3954581</t>
+          <t>C246013</t>
         </is>
       </c>
       <c r="P38" s="16" t="inlineStr">
@@ -3847,17 +3847,17 @@
       </c>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H39" s="17" t="inlineStr">
         <is>
-          <t>ERA-3AEB9762V</t>
+          <t>RT0603BRD0797K6L</t>
         </is>
       </c>
       <c r="I39" s="17" t="inlineStr">
         <is>
-          <t>저항 97.6 kΩ 1% 0603 (UVLO/OVP) [LCSC: 0.1 % 25 ppm (1 %형 LCSC에 없음, 더 좋음)]</t>
+          <t>저항 97.6 kΩ 0.1% 25ppm 0603 (UVLO/OVP) [LCSC: 0.1 % 25 ppm (1 %형 LCSC에 없음, 더 좋음)]</t>
         </is>
       </c>
       <c r="J39" s="19" t="n">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="O39" s="16" t="inlineStr">
         <is>
-          <t>C2074558</t>
+          <t>C861608</t>
         </is>
       </c>
       <c r="P39" s="16" t="inlineStr">
@@ -3909,7 +3909,7 @@
       </c>
       <c r="E40" s="16" t="inlineStr">
         <is>
-          <t>36.5k 1%</t>
+          <t>35.7k 1%</t>
         </is>
       </c>
       <c r="F40" s="16" t="inlineStr">
@@ -3924,12 +3924,12 @@
       </c>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>0603WAF3652T5E</t>
+          <t>0603WAF3572T5E</t>
         </is>
       </c>
       <c r="I40" s="17" t="inlineStr">
         <is>
-          <t>저항 36.5 kΩ 1% 0603 (OVP 32.6 V, 복귀 30.1 V — v0.9)</t>
+          <t>저항 35.7 kΩ 1% 0603 (OVP 32.61 V, 복귀 30.14 V — v0.11)</t>
         </is>
       </c>
       <c r="J40" s="19" t="n">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>C23029</t>
+          <t>C23027</t>
         </is>
       </c>
       <c r="P40" s="16" t="inlineStr">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>80.6k 1%</t>
+          <t>82k 1%</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
@@ -3996,12 +3996,12 @@
       </c>
       <c r="H41" s="17" t="inlineStr">
         <is>
-          <t>0603WAF8062T5E</t>
+          <t>0603WAF8202T5E</t>
         </is>
       </c>
       <c r="I41" s="17" t="inlineStr">
         <is>
-          <t>저항 80.6 kΩ 1% 0603 (TPS2660 전류제한 149 mA = 12/R)</t>
+          <t>저항 82 kΩ 1% 0603 (TPS2660 전류제한 명목 146 mA = 12/R)</t>
         </is>
       </c>
       <c r="J41" s="19" t="n">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="O41" s="16" t="inlineStr">
         <is>
-          <t>C23249</t>
+          <t>C23254</t>
         </is>
       </c>
       <c r="P41" s="16" t="inlineStr">
@@ -4649,7 +4649,7 @@
       </c>
       <c r="I50" s="17" t="inlineStr">
         <is>
-          <t>CRCW 2512 10 Ω 1% 1 W (결정 #38: JLC 부품 — 일반형, 서지 시험 T3로 확인) [LCSC: 결정 #38: 일반형 (HP 대신)]</t>
+          <t>CRCW 2512 10 Ω 1% 1 W (결정 #38: JLC 부품 — 일반형, 서지 시험 T3로 확인) [LCSC: 결정 #57: 일반형 5%; 서지 시험 필요]</t>
         </is>
       </c>
       <c r="J50" s="19" t="n">

</xml_diff>